<commit_message>
update 1.4 vocab exports
</commit_message>
<xml_diff>
--- a/storage/app/public/vocabs/fieldscale/1.4/fieldscale_1-4.xlsx
+++ b/storage/app/public/vocabs/fieldscale/1.4/fieldscale_1-4.xlsx
@@ -23,10 +23,10 @@
     <t>uri</t>
   </si>
   <si>
-    <t>hyperlink</t>
-  </si>
-  <si>
     <t>external_uri</t>
+  </si>
+  <si>
+    <t>external_vocab_scheme</t>
   </si>
   <si>
     <t>Facility names</t>

</xml_diff>